<commit_message>
Atualiza resumos e evolucao com nomenclatura Hermes Pardini.
Resumo vira xlsm com Conferido e macro de altura; altas e ebook saem de Exames; RX de punho e idade ossea alinhados a Dra. Julia.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Relatórios/Resumo Relatórios.xlsx
+++ b/Relatórios/Resumo Relatórios.xlsx
@@ -379,7 +379,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabelaRelatorios" displayName="TabelaRelatorios" ref="A2:D56" headerRowCount="1" headerRowDxfId="2" dataDxfId="0" totalsRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabelaRelatorios" displayName="TabelaRelatorios" ref="A2:D62" headerRowCount="1" headerRowDxfId="2" dataDxfId="0" totalsRowDxfId="1">
   <autoFilter ref="A2:D53"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Data" dataDxfId="6"/>
@@ -680,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -720,129 +720,129 @@
     </row>
     <row r="3" ht="14.4" customHeight="1">
       <c r="A3" s="2" t="n">
-        <v>44683</v>
+        <v>44015</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Endocrino</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Dr. Cristiano</t>
+          <t>Dra. Juliana</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Relatório para solicitação de exoma</t>
+          <t>Alta do berçário</t>
         </is>
       </c>
     </row>
     <row r="4" ht="14.4" customHeight="1">
       <c r="A4" s="2" t="n">
-        <v>44916</v>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Endocrino</t>
+        <v>44103</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Dr. Cristiano</t>
+          <t>Dra. Silvania</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Relatório para solicitação de exoma (dez/2022)</t>
+          <t>Alta do CTI pediátrico</t>
         </is>
       </c>
     </row>
     <row r="5" ht="14.4" customHeight="1">
       <c r="A5" s="2" t="n">
-        <v>45473</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Escola</t>
+        <v>44103</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>EMEI Alaíde Lisboa</t>
+          <t>Dra. Silvania</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Relatório individual 1º semestre/2024</t>
+          <t>Alta CTI — enfermagem</t>
         </is>
       </c>
     </row>
     <row r="6" ht="14.4" customHeight="1">
-      <c r="A6" s="7" t="n">
-        <v>45657</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Escola</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>EMEI Alaíde Lisboa</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Relatório individual 2º semestre/2024</t>
+      <c r="A6" s="2" t="n">
+        <v>44105</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Dra. Raquel</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Alta da pediatria</t>
         </is>
       </c>
     </row>
     <row r="7" ht="14.4" customHeight="1">
-      <c r="A7" s="7" t="n">
-        <v>45838</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Escola</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>EMEI Alaíde Lisboa</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Relatório individual 1º semestre/2025</t>
+      <c r="A7" s="2" t="n">
+        <v>44683</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Endocrino</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Dr. Cristiano</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Relatório para solicitação de exoma</t>
         </is>
       </c>
     </row>
     <row r="8" ht="14.4" customHeight="1">
       <c r="A8" s="2" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Escola</t>
+        <v>44916</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Endocrino</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>EMEI Alaíde Lisboa</t>
+          <t>Dr. Cristiano</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Pauta de observação EI 5/6 anos — 1º período</t>
+          <t>Relatório para solicitação de exoma (dez/2022)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="14.4" customHeight="1">
       <c r="A9" s="2" t="n">
-        <v>46203</v>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
+        <v>45473</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Escola</t>
         </is>
@@ -854,943 +854,1063 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Pauta de observação EI 5/6 anos — 1º semestre</t>
+          <t>Relatório individual 1º semestre/2024</t>
         </is>
       </c>
     </row>
     <row r="10" ht="14.4" customHeight="1">
-      <c r="A10" s="2" t="n">
-        <v>44384</v>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Fisioterapia</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Silvia Figueiredo</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Relatório de sessões (DNPM / hemorragia grau III)</t>
+      <c r="A10" s="7" t="n">
+        <v>45657</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Escola</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>EMEI Alaíde Lisboa</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Relatório individual 2º semestre/2024</t>
         </is>
       </c>
     </row>
     <row r="11" ht="14.4" customHeight="1">
-      <c r="A11" s="2" t="n">
-        <v>45029</v>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Fisioterapia</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Silvia Figueiredo</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Evolução motora (à neurologista)</t>
+      <c r="A11" s="7" t="n">
+        <v>45838</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Escola</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>EMEI Alaíde Lisboa</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Relatório individual 1º semestre/2025</t>
         </is>
       </c>
     </row>
     <row r="12" ht="14.4" customHeight="1">
       <c r="A12" s="7" t="n">
-        <v>45197</v>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Fisioterapia</t>
+        <v>46022</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Escola</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Silvia Figueiredo</t>
+          <t>EMEI Alaíde Lisboa</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Evolução motora (neurologista)</t>
+          <t>Pauta de observação EI 4/5 anos · 3º trimestre</t>
         </is>
       </c>
     </row>
     <row r="13" ht="14.4" customHeight="1">
       <c r="A13" s="2" t="n">
-        <v>45197</v>
+        <v>46203</v>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Fisioterapia</t>
+          <t>Escola</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Silvia Figueiredo</t>
+          <t>EMEI Alaíde Lisboa</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Relatório de sessões (CASU)</t>
+          <t>Pauta de observação EI 5/6 anos — 1º período</t>
         </is>
       </c>
     </row>
     <row r="14" ht="14.4" customHeight="1">
-      <c r="A14" s="7" t="n">
-        <v>45329</v>
+      <c r="A14" s="2" t="n">
+        <v>46203</v>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Fisioterapia</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Silvia Figueiredo</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Alta supervisionada (neurologista)</t>
+          <t>Escola</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>EMEI Alaíde Lisboa</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Pauta de observação EI 5/6 anos — 1º semestre</t>
         </is>
       </c>
     </row>
     <row r="15" ht="14.4" customHeight="1">
       <c r="A15" s="2" t="n">
+        <v>44384</v>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Silvia Figueiredo</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Relatório de sessões (DNPM / hemorragia grau III)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="14.4" customHeight="1">
+      <c r="A16" s="2" t="n">
+        <v>45029</v>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Silvia Figueiredo</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Evolução motora (à neurologista)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="14.4" customHeight="1">
+      <c r="A17" s="7" t="n">
+        <v>45197</v>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Silvia Figueiredo</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Evolução motora (neurologista)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="14.4" customHeight="1">
+      <c r="A18" s="2" t="n">
+        <v>45197</v>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Silvia Figueiredo</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Relatório de sessões (CASU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="14.4" customHeight="1">
+      <c r="A19" s="7" t="n">
         <v>45329</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Fisioterapia</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Silvia Figueiredo</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Relatório de sessões / alta (CASU)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="14.4" customHeight="1">
-      <c r="A16" s="7" t="n">
-        <v>45544</v>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Fisioterapia</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Silvia Figueiredo</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Reavaliação após alta</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="14.4" customHeight="1">
-      <c r="A17" s="2" t="n">
-        <v>45861</v>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Fisioterapia</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Silvia Figueiredo</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Reavaliação periódica</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="14.4" customHeight="1">
-      <c r="A18" s="7" t="n">
-        <v>45861</v>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Fisioterapia</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Silvia Figueiredo</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Relatório ao educador físico Marlon</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="14.4" customHeight="1">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>Fisioterapia</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Silvia Figueiredo</t>
-        </is>
-      </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Ebook Estimula Bebê (material, não é relatório da Cecília)</t>
+          <t>Alta supervisionada (neurologista)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="14.4" customHeight="1">
       <c r="A20" s="2" t="n">
+        <v>45329</v>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Silvia Figueiredo</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Relatório de sessões / alta (CASU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="14.4" customHeight="1">
+      <c r="A21" s="7" t="n">
+        <v>45544</v>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Silvia Figueiredo</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Reavaliação após alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="14.4" customHeight="1">
+      <c r="A22" s="2" t="n">
+        <v>45861</v>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Silvia Figueiredo</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Reavaliação periódica</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="14.4" customHeight="1">
+      <c r="A23" s="7" t="n">
+        <v>45861</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Silvia Figueiredo</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Relatório ao educador físico Marlon</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="14.4" customHeight="1">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Silvia Figueiredo</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Ebook Estimula Bebê (material, não é relatório da Cecília)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="14.4" customHeight="1">
+      <c r="A25" s="2" t="n">
         <v>44777</v>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Fonoaudiologia</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Viviane Sampaio</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Relatório de acompanhamento (atraso de fala)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="14.4" customHeight="1">
-      <c r="A21" s="2" t="n">
-        <v>44939</v>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>Fonoaudiologia</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Viviane Sampaio</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Relatório de evolução</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="14.4" customHeight="1">
-      <c r="A22" s="7" t="n">
-        <v>44956</v>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Fonoaudiologia</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Fernanda Alvarenga</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Avaliação fonoaudiológica (Travessia)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="14.4" customHeight="1">
-      <c r="A23" s="2" t="n">
-        <v>45530</v>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Fonoaudiologia</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Viviane Sampaio</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Relatório de acompanhamento</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="14.4" customHeight="1">
-      <c r="A24" s="7" t="n">
-        <v>45623</v>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>Fonoaudiologia</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Fernanda Alvarenga</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Acompanhamento (Travessia)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="14.4" customHeight="1">
-      <c r="A25" s="7" t="n">
-        <v>45689</v>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>Fonoaudiologia</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Viviane Sampaio</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>Relatório de acompanhamento</t>
         </is>
       </c>
     </row>
     <row r="26" ht="14.4" customHeight="1">
       <c r="A26" s="2" t="n">
+        <v>44939</v>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Fonoaudiologia</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Viviane Sampaio</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Relatório de evolução</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="14.4" customHeight="1">
+      <c r="A27" s="7" t="n">
+        <v>44956</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Fonoaudiologia</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Fernanda Alvarenga</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Avaliação fonoaudiológica (Travessia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="14.4" customHeight="1">
+      <c r="A28" s="2" t="n">
+        <v>45530</v>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Fonoaudiologia</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Viviane Sampaio</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Relatório de acompanhamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="14.4" customHeight="1">
+      <c r="A29" s="7" t="n">
+        <v>45623</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Fonoaudiologia</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Fernanda Alvarenga</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>Acompanhamento (Travessia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="14.4" customHeight="1">
+      <c r="A30" s="7" t="n">
+        <v>45624</v>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Fonoaudiologia</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Fernanda Alvarenga</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Relato em fonoaudiologia (Travessia; ABFW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="14.4" customHeight="1">
+      <c r="A31" s="7" t="n">
+        <v>45689</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Fonoaudiologia</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Viviane Sampaio</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>Relatório de acompanhamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="14.4" customHeight="1">
+      <c r="A32" s="2" t="n">
         <v>45870</v>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Fonoaudiologia</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Viviane Sampaio</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>Relatório de alta/evolução</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="14.4" customHeight="1">
-      <c r="A27" s="2" t="n">
+    <row r="33" ht="14.4" customHeight="1">
+      <c r="A33" s="2" t="n">
         <v>45390</v>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Funcional</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Marlon Costa</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>Relatório de educação física</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="14.4" customHeight="1">
-      <c r="A28" s="7" t="n">
-        <v>45524</v>
-      </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>Funcional</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Marlon Costa</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>Avaliação Funcional Kids</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="14.4" customHeight="1">
-      <c r="A29" s="2" t="n">
-        <v>45835</v>
-      </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>Funcional</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Marlon Costa</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Avaliação Funcional Kids</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="14.4" customHeight="1">
-      <c r="A30" s="2" t="n">
-        <v>46139</v>
-      </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>Funcional</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Marlon Costa</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>Avaliação Funcional Kids</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="14.4" customHeight="1">
-      <c r="A31" s="2" t="n">
-        <v>45818</v>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Genética</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Dra. Milena</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Pedido/resumo: exoma + CNV + DNA mitocondrial</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="14.4" customHeight="1">
-      <c r="A32" s="7" t="n">
-        <v>45895</v>
-      </c>
-      <c r="B32" s="13" t="inlineStr">
-        <is>
-          <t>Genética</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Dra. Milena</t>
-        </is>
-      </c>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>Relatório clínico (para Dr. Guilherme)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="14.4" customHeight="1">
-      <c r="A33" s="7" t="n">
-        <v>45376</v>
-      </c>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>Natação</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>Connect Acqua Kids</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Gestão de desenvolvimento (jan–mar/2024)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="14.4" customHeight="1">
       <c r="A34" s="7" t="n">
-        <v>45454</v>
-      </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>Natação</t>
+        <v>45524</v>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Connect Acqua Kids</t>
+          <t>Marlon Costa</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Gestão de desenvolvimento (mar–mai/2024)</t>
+          <t>Avaliação Funcional Kids</t>
         </is>
       </c>
     </row>
     <row r="35" ht="14.4" customHeight="1">
       <c r="A35" s="2" t="n">
-        <v>45548</v>
-      </c>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>Natação</t>
+        <v>45835</v>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Connect Acqua Kids</t>
+          <t>Marlon Costa</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Gestão de desenvolvimento (jun–ago/2024)</t>
+          <t>Avaliação Funcional Kids</t>
         </is>
       </c>
     </row>
     <row r="36" ht="14.4" customHeight="1">
       <c r="A36" s="2" t="n">
-        <v>45627</v>
-      </c>
-      <c r="B36" s="14" t="inlineStr">
-        <is>
-          <t>Natação</t>
+        <v>46139</v>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>Funcional</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Connect Acqua Kids</t>
+          <t>Marlon Costa</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Gestão de desenvolvimento (frequência)</t>
+          <t>Avaliação Funcional Kids</t>
         </is>
       </c>
     </row>
     <row r="37" ht="14.4" customHeight="1">
-      <c r="A37" s="7" t="n">
-        <v>45809</v>
-      </c>
-      <c r="B37" s="14" t="inlineStr">
-        <is>
-          <t>Natação</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>Connect Acqua Kids</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>Gestão de desenvolvimento (mar–mai/2025)</t>
+      <c r="A37" s="2" t="n">
+        <v>45818</v>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Genética</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Dra. Milena</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Pedido/resumo: exoma + CNV + DNA mitocondrial</t>
         </is>
       </c>
     </row>
     <row r="38" ht="14.4" customHeight="1">
       <c r="A38" s="7" t="n">
-        <v>46141</v>
-      </c>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>Natação</t>
+        <v>45895</v>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Genética</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>Connect Acqua Kids</t>
+          <t>Dra. Milena</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>Relatório de acompanhamento (Acqua Aprendizado)</t>
+          <t>Relatório clínico (para Dr. Guilherme)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="14.4" customHeight="1">
       <c r="A39" s="7" t="n">
-        <v>44455</v>
-      </c>
-      <c r="B39" s="15" t="inlineStr">
-        <is>
-          <t>Neuro</t>
+        <v>45376</v>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>Natação</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Dra. Luciana Gauzzi</t>
+          <t>Connect Acqua Kids</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>Relatório neurológico (hidrocefalia, DVP, atraso DNPM)</t>
+          <t>Gestão de desenvolvimento (jan–mar/2024)</t>
         </is>
       </c>
     </row>
     <row r="40" ht="14.4" customHeight="1">
-      <c r="A40" s="2" t="n">
-        <v>45699</v>
-      </c>
-      <c r="B40" s="15" t="inlineStr">
-        <is>
-          <t>Neuro</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Dra. Luciana Gauzzi</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Relatório de transferência</t>
+      <c r="A40" s="7" t="n">
+        <v>45454</v>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>Natação</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Connect Acqua Kids</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Gestão de desenvolvimento (mar–mai/2024)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="14.4" customHeight="1">
-      <c r="A41" s="7" t="n">
-        <v>44212</v>
-      </c>
-      <c r="B41" s="16" t="inlineStr">
-        <is>
-          <t>Oftalmologia</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>Dra. Débora Pinheiro</t>
-        </is>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>Relatório oftalmológico</t>
+      <c r="A41" s="2" t="n">
+        <v>45548</v>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>Natação</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Connect Acqua Kids</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Gestão de desenvolvimento (jun–ago/2024)</t>
         </is>
       </c>
     </row>
     <row r="42" ht="14.4" customHeight="1">
       <c r="A42" s="2" t="n">
-        <v>44816</v>
-      </c>
-      <c r="B42" s="16" t="inlineStr">
-        <is>
-          <t>Oftalmologia</t>
+        <v>45627</v>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>Natação</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Dra. Débora Pinheiro</t>
+          <t>Connect Acqua Kids</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Relatório oftalmológico</t>
+          <t>Gestão de desenvolvimento (frequência)</t>
         </is>
       </c>
     </row>
     <row r="43" ht="14.4" customHeight="1">
       <c r="A43" s="7" t="n">
-        <v>44965</v>
-      </c>
-      <c r="B43" s="16" t="inlineStr">
-        <is>
-          <t>Oftalmologia</t>
+        <v>45809</v>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>Natação</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Dra. Débora Pinheiro</t>
+          <t>Connect Acqua Kids</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>Relatório oftalmológico</t>
+          <t>Gestão de desenvolvimento (mar–mai/2025)</t>
         </is>
       </c>
     </row>
     <row r="44" ht="14.4" customHeight="1">
       <c r="A44" s="7" t="n">
-        <v>45260</v>
-      </c>
-      <c r="B44" s="16" t="inlineStr">
+        <v>46141</v>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Natação</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Connect Acqua Kids</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Relatório de acompanhamento (Acqua Aprendizado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="14.4" customHeight="1">
+      <c r="A45" s="7" t="n">
+        <v>44455</v>
+      </c>
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>Neuro</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Dra. Luciana Gauzzi</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Relatório neurológico (hidrocefalia, DVP, atraso DNPM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="14.4" customHeight="1">
+      <c r="A46" s="2" t="n">
+        <v>45699</v>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>Neuro</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Dra. Luciana Gauzzi</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Relatório de transferência</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="14.4" customHeight="1">
+      <c r="A47" s="7" t="n">
+        <v>44212</v>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
         <is>
           <t>Oftalmologia</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
+      <c r="C47" s="8" t="inlineStr">
         <is>
           <t>Dra. Débora Pinheiro</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr">
-        <is>
-          <t>Relatório oftalmológico (óculos e oclusão)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="14.4" customHeight="1">
-      <c r="A45" s="2" t="n">
-        <v>45910</v>
-      </c>
-      <c r="B45" s="17" t="inlineStr">
-        <is>
-          <t>Pedagogia</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Rosemary Albergaria</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>Relatório pedagógico (atenção e autonomia)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="14.4" customHeight="1">
-      <c r="A46" s="7" t="n">
-        <v>45844</v>
-      </c>
-      <c r="B46" s="18" t="inlineStr">
-        <is>
-          <t>Psicologia</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>Ana Clara Moreira</t>
-        </is>
-      </c>
-      <c r="D46" s="9" t="inlineStr">
-        <is>
-          <t>Relatório psicológico (Ampliar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="14.4" customHeight="1">
-      <c r="A47" s="2" t="n">
-        <v>44490</v>
-      </c>
-      <c r="B47" s="19" t="inlineStr">
-        <is>
-          <t>TO</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>Aline Serva</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>Bayley III</t>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Relatório oftalmológico</t>
         </is>
       </c>
     </row>
     <row r="48" ht="14.4" customHeight="1">
-      <c r="A48" s="7" t="n">
-        <v>44686</v>
-      </c>
-      <c r="B48" s="19" t="inlineStr">
-        <is>
-          <t>TO</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t>Aline Serva</t>
-        </is>
-      </c>
-      <c r="D48" s="9" t="inlineStr">
-        <is>
-          <t>Bayley III</t>
+      <c r="A48" s="2" t="n">
+        <v>44816</v>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>Oftalmologia</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Dra. Débora Pinheiro</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Relatório oftalmológico</t>
         </is>
       </c>
     </row>
     <row r="49" ht="14.4" customHeight="1">
       <c r="A49" s="7" t="n">
-        <v>44927</v>
-      </c>
-      <c r="B49" s="19" t="inlineStr">
-        <is>
-          <t>TO</t>
+        <v>44965</v>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>Oftalmologia</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Aline Serva</t>
+          <t>Dra. Débora Pinheiro</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>Relatório de TO para escola</t>
+          <t>Relatório oftalmológico</t>
         </is>
       </c>
     </row>
     <row r="50" ht="14.4" customHeight="1">
-      <c r="A50" s="2" t="n">
-        <v>45671</v>
-      </c>
-      <c r="B50" s="19" t="inlineStr">
-        <is>
-          <t>TO</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Carol Ribeiro</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Reavaliação de terapia ocupacional</t>
+      <c r="A50" s="7" t="n">
+        <v>45260</v>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>Oftalmologia</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Dra. Débora Pinheiro</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>Relatório oftalmológico (óculos e oclusão)</t>
         </is>
       </c>
     </row>
     <row r="51" ht="14.4" customHeight="1">
-      <c r="A51" s="7" t="n">
-        <v>44550</v>
-      </c>
-      <c r="B51" s="20" t="inlineStr">
-        <is>
-          <t>TO Visão</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>Aline Brandão</t>
-        </is>
-      </c>
-      <c r="D51" s="9" t="inlineStr">
-        <is>
-          <t>Avaliação da visão funcional (AVIF)</t>
+      <c r="A51" s="2" t="n">
+        <v>45910</v>
+      </c>
+      <c r="B51" s="17" t="inlineStr">
+        <is>
+          <t>Pedagogia</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Rosemary Albergaria</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Relatório pedagógico (atenção e autonomia)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n">
-        <v>44789</v>
-      </c>
-      <c r="B52" s="20" t="inlineStr">
-        <is>
-          <t>TO Visão</t>
+        <v>45844</v>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>Psicologia</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>Aline Brandão</t>
+          <t>Ana Clara Moreira</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Reavaliação da visão funcional (AVIF 85/100)</t>
+          <t>Relatório psicológico (Ampliar)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>44956</v>
-      </c>
-      <c r="B53" s="20" t="inlineStr">
-        <is>
-          <t>TO Visão</t>
+        <v>44490</v>
+      </c>
+      <c r="B53" s="19" t="inlineStr">
+        <is>
+          <t>TO</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Aline Brandão</t>
+          <t>Aline Serva</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Declaração de habilitação visual para a EMEI</t>
+          <t>Bayley III</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
-        <v>45017</v>
-      </c>
-      <c r="B54" s="20" t="inlineStr">
-        <is>
-          <t>TO Visão</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Aline Brandão</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Relatório para a CASU</t>
+      <c r="A54" s="7" t="n">
+        <v>44686</v>
+      </c>
+      <c r="B54" s="19" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>Aline Serva</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>Bayley III</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n">
-        <v>45017</v>
-      </c>
-      <c r="B55" s="20" t="inlineStr">
-        <is>
-          <t>TO Visão</t>
+        <v>44927</v>
+      </c>
+      <c r="B55" s="19" t="inlineStr">
+        <is>
+          <t>TO</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Aline Brandão</t>
+          <t>Aline Serva</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>Relatório para a EMEI</t>
+          <t>Relatório de TO para escola</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
+        <v>45671</v>
+      </c>
+      <c r="B56" s="19" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Carol Ribeiro</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Reavaliação de terapia ocupacional</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="n">
+        <v>44550</v>
+      </c>
+      <c r="B57" s="20" t="inlineStr">
+        <is>
+          <t>TO Visão</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>Aline Brandão</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>Avaliação da visão funcional (AVIF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="n">
+        <v>44789</v>
+      </c>
+      <c r="B58" s="20" t="inlineStr">
+        <is>
+          <t>TO Visão</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Aline Brandão</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>Reavaliação da visão funcional (AVIF 85/100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>44956</v>
+      </c>
+      <c r="B59" s="20" t="inlineStr">
+        <is>
+          <t>TO Visão</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Aline Brandão</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Declaração de habilitação visual para a EMEI</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>45017</v>
+      </c>
+      <c r="B60" s="20" t="inlineStr">
+        <is>
+          <t>TO Visão</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Aline Brandão</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Relatório para a CASU</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="n">
+        <v>45017</v>
+      </c>
+      <c r="B61" s="20" t="inlineStr">
+        <is>
+          <t>TO Visão</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>Aline Brandão</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>Relatório para a EMEI</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
         <v>45261</v>
       </c>
-      <c r="B56" s="20" t="inlineStr">
+      <c r="B62" s="20" t="inlineStr">
         <is>
           <t>TO Visão</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Aline Brandão</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>Reavaliação AVIF (93/100)</t>
         </is>

</xml_diff>